<commit_message>
Updated changes as per report analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30546FB0-A7E3-4EB5-99E7-8D184D9B803A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5284B5BB-16D9-4603-8806-FB224E9E3A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
@@ -604,11 +604,11 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
+      <c r="B3" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated changes as per analysis report
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798419C6-67D0-40EA-99DB-446C44FBB53B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB15489-1E26-4B25-8F25-CA7DA7A46F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
@@ -262,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -285,8 +285,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -604,7 +602,7 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
@@ -744,7 +742,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B16" s="12"/>
+      <c r="B16" s="10"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="5"/>
@@ -782,7 +780,7 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>29</v>
       </c>
       <c r="C2" t="s">
@@ -793,7 +791,7 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>31</v>
       </c>
       <c r="C3" t="s">
@@ -804,7 +802,7 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -837,7 +835,7 @@
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="11" t="s">
         <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -848,7 +846,7 @@
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="11" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -859,7 +857,7 @@
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="11" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -1101,15 +1099,15 @@
       <c r="B14" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="5">
         <v>15000</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C15" s="11"/>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C16" s="11"/>
+      <c r="C16" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1481,7 +1479,7 @@
   <cols>
     <col min="1" max="1" width="23.109375" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="3" width="60.6640625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1023 1026:2046 2049:3072 3075:4095 4098:5118 5121:6144 6147:7167 7170:8190 8193:9216 9219:10239 10242:11262 11265:12288 12291:13311 13314:14334 14337:15360 15363:16383" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -6986,7 +6984,7 @@
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="7"/>
@@ -7010,7 +7008,7 @@
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" s="8"/>
@@ -7022,7 +7020,7 @@
       <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7">
         <v>365</v>
       </c>
       <c r="D7" s="9"/>
@@ -7034,7 +7032,7 @@
       <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="9"/>
@@ -7046,7 +7044,7 @@
       <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="9"/>
@@ -7058,7 +7056,7 @@
       <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="9"/>
@@ -7070,7 +7068,7 @@
       <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="9"/>
@@ -7082,7 +7080,7 @@
       <c r="B12" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="5" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="9"/>
@@ -7094,7 +7092,7 @@
       <c r="B13" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="9"/>
@@ -7106,7 +7104,7 @@
       <c r="B14" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="9"/>

</xml_diff>

<commit_message>
Changes as per analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C2F22D-A80F-4A4A-BED7-D7934971F184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3232C1BC-B0C0-4C5A-A076-7ED811AB15E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
@@ -193,7 +193,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,12 +229,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF202124"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
-    <font>
       <sz val="7"/>
       <color rgb="FF202124"/>
       <name val="Consolas"/>
@@ -262,7 +256,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -286,7 +280,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -568,12 +561,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D795F61-CC1F-4314-B1D8-0852B981BA18}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -591,8 +584,8 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
+      <c r="B2" s="10" t="s">
+        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -602,22 +595,22 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>34</v>
+      <c r="B3" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
+      <c r="B4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -625,10 +618,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -636,43 +629,43 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3">
-        <v>0</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="3">
-        <v>365</v>
+      <c r="B7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
-        <v>16</v>
+      <c r="B8" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
+      <c r="B9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -742,14 +735,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B16" s="10"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="5"/>
+      <c r="B16" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{7EE9E90B-967F-44F2-8381-163CD7361D89}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{E1F97CBA-2299-4C5C-9A3F-BE0AC4C69AE9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -780,7 +770,7 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>29</v>
       </c>
       <c r="C2" t="s">
@@ -791,7 +781,7 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>31</v>
       </c>
       <c r="C3" t="s">
@@ -802,7 +792,7 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -835,7 +825,7 @@
       <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -846,7 +836,7 @@
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>34</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -857,7 +847,7 @@
       <c r="A9" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="3" t="s">

</xml_diff>

<commit_message>
Updated test cases and added new steps as per report analysis
</commit_message>
<xml_diff>
--- a/src/main/resources/Program_Field_Values.xlsx
+++ b/src/main/resources/Program_Field_Values.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3232C1BC-B0C0-4C5A-A076-7ED811AB15E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3229B9D4-1230-4DCB-8AEC-916D61FB28D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="3" r:id="rId1"/>
     <sheet name="Creation_v" sheetId="7" r:id="rId2"/>
     <sheet name="AnnouncementCreation_v" sheetId="8" r:id="rId3"/>
-    <sheet name="Creation1" sheetId="4" r:id="rId4"/>
-    <sheet name="CreationWithoutDescription" sheetId="5" r:id="rId5"/>
-    <sheet name="CreationForAnnouncement" sheetId="6" r:id="rId6"/>
+    <sheet name="AnnouncementCreationCalendar_v" sheetId="9" r:id="rId4"/>
+    <sheet name="Creation1" sheetId="4" r:id="rId5"/>
+    <sheet name="CreationWithoutDescription" sheetId="5" r:id="rId6"/>
+    <sheet name="CreationForAnnouncement" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="54">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -1109,6 +1110,163 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E032D7E5-9EEB-448F-87FD-9AA9E6F783C2}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="5">
+        <v>15000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08A1553C-F7A5-4DD1-9371-6162AF52CB21}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1290,7 +1448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A50E0F2B-3F25-474D-88CC-BA332CE28F6A}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1462,7 +1620,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D0851E1-AAF8-44F9-AFC4-73C66EBF0B6F}">
   <dimension ref="A1:XFC15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>